<commit_message>
Auto update wallet tracker 2026-08-05 08:59 UTC
</commit_message>
<xml_diff>
--- a/data/theo_doi_vi.xlsx
+++ b/data/theo_doi_vi.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.####"/>
     <numFmt numFmtId="165" formatCode="+#,##0.####;-#,##0.####;0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +37,16 @@
     <font>
       <name val="Arial"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +57,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -91,6 +111,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -458,13 +484,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,6 +516,16 @@
           <t>Chênh lệch</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>05/08/2026 15:59</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Chênh lệch</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -504,6 +542,12 @@
         <v>6254146.877</v>
       </c>
       <c r="D2" s="5" t="n"/>
+      <c r="E2" s="4" t="n">
+        <v>6238546.7092</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>-15600.1678</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -520,6 +564,12 @@
         <v>4593414.2832</v>
       </c>
       <c r="D3" s="5" t="n"/>
+      <c r="E3" s="4" t="n">
+        <v>4593414.2832</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -536,6 +586,12 @@
         <v>4032682.9341</v>
       </c>
       <c r="D4" s="5" t="n"/>
+      <c r="E4" s="4" t="n">
+        <v>4032682.9341</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -552,6 +608,12 @@
         <v>4000000</v>
       </c>
       <c r="D5" s="5" t="n"/>
+      <c r="E5" s="4" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -568,6 +630,12 @@
         <v>3663634.4136</v>
       </c>
       <c r="D6" s="5" t="n"/>
+      <c r="E6" s="4" t="n">
+        <v>3663634.4136</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -584,6 +652,12 @@
         <v>3628524.82</v>
       </c>
       <c r="D7" s="5" t="n"/>
+      <c r="E7" s="4" t="n">
+        <v>3628524.82</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -600,6 +674,12 @@
         <v>2743926.9899</v>
       </c>
       <c r="D8" s="5" t="n"/>
+      <c r="E8" s="4" t="n">
+        <v>2743926.9899</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -616,6 +696,12 @@
         <v>2407572.5386</v>
       </c>
       <c r="D9" s="5" t="n"/>
+      <c r="E9" s="4" t="n">
+        <v>2407572.5386</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -632,6 +718,12 @@
         <v>2000000.0012</v>
       </c>
       <c r="D10" s="5" t="n"/>
+      <c r="E10" s="4" t="n">
+        <v>2000000.0012</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -648,6 +740,12 @@
         <v>2000000</v>
       </c>
       <c r="D11" s="5" t="n"/>
+      <c r="E11" s="4" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -664,6 +762,12 @@
         <v>1938773.4789</v>
       </c>
       <c r="D12" s="5" t="n"/>
+      <c r="E12" s="4" t="n">
+        <v>1938773.4789</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -680,6 +784,12 @@
         <v>1810914.2302</v>
       </c>
       <c r="D13" s="5" t="n"/>
+      <c r="E13" s="4" t="n">
+        <v>1810914.2302</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -696,6 +806,12 @@
         <v>1663791.3571</v>
       </c>
       <c r="D14" s="5" t="n"/>
+      <c r="E14" s="4" t="n">
+        <v>1663791.3571</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -712,6 +828,12 @@
         <v>1501314.8913</v>
       </c>
       <c r="D15" s="5" t="n"/>
+      <c r="E15" s="4" t="n">
+        <v>1501314.8913</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -728,6 +850,12 @@
         <v>1236777.8944</v>
       </c>
       <c r="D16" s="5" t="n"/>
+      <c r="E16" s="4" t="n">
+        <v>1236777.8944</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -744,6 +872,12 @@
         <v>1200000</v>
       </c>
       <c r="D17" s="5" t="n"/>
+      <c r="E17" s="4" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -760,6 +894,12 @@
         <v>1178546.0449</v>
       </c>
       <c r="D18" s="5" t="n"/>
+      <c r="E18" s="4" t="n">
+        <v>1178546.0449</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -776,6 +916,12 @@
         <v>1173068.8403</v>
       </c>
       <c r="D19" s="5" t="n"/>
+      <c r="E19" s="4" t="n">
+        <v>1173068.8403</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -792,6 +938,12 @@
         <v>1075254.7301</v>
       </c>
       <c r="D20" s="5" t="n"/>
+      <c r="E20" s="4" t="n">
+        <v>1075254.7301</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -808,6 +960,12 @@
         <v>1070173.9749</v>
       </c>
       <c r="D21" s="5" t="n"/>
+      <c r="E21" s="4" t="n">
+        <v>1070173.9749</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -824,6 +982,12 @@
         <v>1030000</v>
       </c>
       <c r="D22" s="5" t="n"/>
+      <c r="E22" s="4" t="n">
+        <v>1030000</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -840,6 +1004,12 @@
         <v>1027286.3894</v>
       </c>
       <c r="D23" s="5" t="n"/>
+      <c r="E23" s="4" t="n">
+        <v>1027286.3894</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -856,6 +1026,12 @@
         <v>1023082.1439</v>
       </c>
       <c r="D24" s="5" t="n"/>
+      <c r="E24" s="4" t="n">
+        <v>1023082.1439</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -872,6 +1048,12 @@
         <v>1012395.8946</v>
       </c>
       <c r="D25" s="5" t="n"/>
+      <c r="E25" s="4" t="n">
+        <v>1012395.8946</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -888,6 +1070,12 @@
         <v>1009987.2763</v>
       </c>
       <c r="D26" s="5" t="n"/>
+      <c r="E26" s="4" t="n">
+        <v>1009987.2763</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -904,6 +1092,12 @@
         <v>1006825.8922</v>
       </c>
       <c r="D27" s="5" t="n"/>
+      <c r="E27" s="4" t="n">
+        <v>1006825.8922</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -920,6 +1114,12 @@
         <v>1000000</v>
       </c>
       <c r="D28" s="5" t="n"/>
+      <c r="E28" s="4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -936,6 +1136,12 @@
         <v>1000000</v>
       </c>
       <c r="D29" s="5" t="n"/>
+      <c r="E29" s="4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -952,6 +1158,12 @@
         <v>998014.552</v>
       </c>
       <c r="D30" s="5" t="n"/>
+      <c r="E30" s="4" t="n">
+        <v>998014.552</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -968,6 +1180,12 @@
         <v>990000</v>
       </c>
       <c r="D31" s="5" t="n"/>
+      <c r="E31" s="4" t="n">
+        <v>990000</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -984,6 +1202,12 @@
         <v>979187.2334</v>
       </c>
       <c r="D32" s="5" t="n"/>
+      <c r="E32" s="4" t="n">
+        <v>979187.2334</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1000,6 +1224,12 @@
         <v>889548.5399</v>
       </c>
       <c r="D33" s="5" t="n"/>
+      <c r="E33" s="4" t="n">
+        <v>889548.5399</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1016,6 +1246,12 @@
         <v>887524.782</v>
       </c>
       <c r="D34" s="5" t="n"/>
+      <c r="E34" s="4" t="n">
+        <v>887524.782</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1032,6 +1268,12 @@
         <v>879501.0418</v>
       </c>
       <c r="D35" s="5" t="n"/>
+      <c r="E35" s="4" t="n">
+        <v>879501.0418</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1048,6 +1290,12 @@
         <v>862367.0839</v>
       </c>
       <c r="D36" s="5" t="n"/>
+      <c r="E36" s="4" t="n">
+        <v>862367.0839</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1064,6 +1312,12 @@
         <v>838549.1449</v>
       </c>
       <c r="D37" s="5" t="n"/>
+      <c r="E37" s="4" t="n">
+        <v>838549.1449</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1080,6 +1334,12 @@
         <v>836992.2512000001</v>
       </c>
       <c r="D38" s="5" t="n"/>
+      <c r="E38" s="4" t="n">
+        <v>836992.2512000001</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1096,6 +1356,12 @@
         <v>834355.5257</v>
       </c>
       <c r="D39" s="5" t="n"/>
+      <c r="E39" s="4" t="n">
+        <v>834355.5257</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1112,6 +1378,12 @@
         <v>823353.5943</v>
       </c>
       <c r="D40" s="5" t="n"/>
+      <c r="E40" s="4" t="n">
+        <v>823353.5943</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1128,6 +1400,12 @@
         <v>809555.4168</v>
       </c>
       <c r="D41" s="5" t="n"/>
+      <c r="E41" s="4" t="n">
+        <v>809555.4168</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1144,6 +1422,12 @@
         <v>799900.5672</v>
       </c>
       <c r="D42" s="5" t="n"/>
+      <c r="E42" s="4" t="n">
+        <v>799900.5672</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1160,6 +1444,12 @@
         <v>763127.9248</v>
       </c>
       <c r="D43" s="5" t="n"/>
+      <c r="E43" s="4" t="n">
+        <v>763127.9248</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1176,6 +1466,12 @@
         <v>747868.0344</v>
       </c>
       <c r="D44" s="5" t="n"/>
+      <c r="E44" s="4" t="n">
+        <v>747868.0344</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1192,6 +1488,12 @@
         <v>732703.1313</v>
       </c>
       <c r="D45" s="5" t="n"/>
+      <c r="E45" s="4" t="n">
+        <v>732703.1313</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1208,6 +1510,12 @@
         <v>725096.5494</v>
       </c>
       <c r="D46" s="5" t="n"/>
+      <c r="E46" s="4" t="n">
+        <v>725096.5494</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1224,6 +1532,12 @@
         <v>711759.0045</v>
       </c>
       <c r="D47" s="5" t="n"/>
+      <c r="E47" s="4" t="n">
+        <v>711759.0045</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1240,6 +1554,12 @@
         <v>693657.6485</v>
       </c>
       <c r="D48" s="5" t="n"/>
+      <c r="E48" s="4" t="n">
+        <v>693657.6485</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1256,6 +1576,12 @@
         <v>672356.3260999999</v>
       </c>
       <c r="D49" s="5" t="n"/>
+      <c r="E49" s="4" t="n">
+        <v>672356.3260999999</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1272,6 +1598,12 @@
         <v>645576.1191</v>
       </c>
       <c r="D50" s="5" t="n"/>
+      <c r="E50" s="4" t="n">
+        <v>645576.1191</v>
+      </c>
+      <c r="F50" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1288,6 +1620,12 @@
         <v>645051.7397</v>
       </c>
       <c r="D51" s="5" t="n"/>
+      <c r="E51" s="4" t="n">
+        <v>645051.7397</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1304,6 +1642,12 @@
         <v>634607.2181000001</v>
       </c>
       <c r="D52" s="5" t="n"/>
+      <c r="E52" s="4" t="n">
+        <v>634607.2181000001</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1320,6 +1664,12 @@
         <v>620661.4845</v>
       </c>
       <c r="D53" s="5" t="n"/>
+      <c r="E53" s="4" t="n">
+        <v>620661.4845</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1336,6 +1686,12 @@
         <v>618815.814</v>
       </c>
       <c r="D54" s="5" t="n"/>
+      <c r="E54" s="4" t="n">
+        <v>618815.814</v>
+      </c>
+      <c r="F54" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1352,6 +1708,12 @@
         <v>577999.0600000001</v>
       </c>
       <c r="D55" s="5" t="n"/>
+      <c r="E55" s="4" t="n">
+        <v>577999.0600000001</v>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1368,6 +1730,12 @@
         <v>574396.1581</v>
       </c>
       <c r="D56" s="5" t="n"/>
+      <c r="E56" s="4" t="n">
+        <v>574396.1581</v>
+      </c>
+      <c r="F56" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1384,6 +1752,12 @@
         <v>543641.1091999999</v>
       </c>
       <c r="D57" s="5" t="n"/>
+      <c r="E57" s="4" t="n">
+        <v>543641.1091999999</v>
+      </c>
+      <c r="F57" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1400,6 +1774,12 @@
         <v>540799.1483999999</v>
       </c>
       <c r="D58" s="5" t="n"/>
+      <c r="E58" s="4" t="n">
+        <v>540799.1483999999</v>
+      </c>
+      <c r="F58" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1416,6 +1796,12 @@
         <v>522769.5865</v>
       </c>
       <c r="D59" s="5" t="n"/>
+      <c r="E59" s="4" t="n">
+        <v>522769.5865</v>
+      </c>
+      <c r="F59" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1432,6 +1818,12 @@
         <v>514620.6938</v>
       </c>
       <c r="D60" s="5" t="n"/>
+      <c r="E60" s="4" t="n">
+        <v>514620.6938</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1448,6 +1840,12 @@
         <v>502486.445</v>
       </c>
       <c r="D61" s="5" t="n"/>
+      <c r="E61" s="4" t="n">
+        <v>502486.445</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1464,6 +1862,12 @@
         <v>500000.0059</v>
       </c>
       <c r="D62" s="5" t="n"/>
+      <c r="E62" s="4" t="n">
+        <v>500000.0059</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1480,6 +1884,12 @@
         <v>496416.2686</v>
       </c>
       <c r="D63" s="5" t="n"/>
+      <c r="E63" s="4" t="n">
+        <v>496416.2686</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1496,6 +1906,12 @@
         <v>493196.1109</v>
       </c>
       <c r="D64" s="5" t="n"/>
+      <c r="E64" s="4" t="n">
+        <v>493196.1109</v>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1512,6 +1928,12 @@
         <v>492785.4309</v>
       </c>
       <c r="D65" s="5" t="n"/>
+      <c r="E65" s="4" t="n">
+        <v>492785.4309</v>
+      </c>
+      <c r="F65" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1528,6 +1950,12 @@
         <v>485670.7376</v>
       </c>
       <c r="D66" s="5" t="n"/>
+      <c r="E66" s="4" t="n">
+        <v>485670.7376</v>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1544,6 +1972,12 @@
         <v>479895.4935</v>
       </c>
       <c r="D67" s="5" t="n"/>
+      <c r="E67" s="4" t="n">
+        <v>479895.4935</v>
+      </c>
+      <c r="F67" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1560,6 +1994,12 @@
         <v>478481.1661</v>
       </c>
       <c r="D68" s="5" t="n"/>
+      <c r="E68" s="4" t="n">
+        <v>478481.1661</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1576,6 +2016,12 @@
         <v>475707.078</v>
       </c>
       <c r="D69" s="5" t="n"/>
+      <c r="E69" s="4" t="n">
+        <v>475707.078</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1592,6 +2038,12 @@
         <v>464907.3106</v>
       </c>
       <c r="D70" s="5" t="n"/>
+      <c r="E70" s="4" t="n">
+        <v>464907.3106</v>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1608,6 +2060,12 @@
         <v>456856.3119</v>
       </c>
       <c r="D71" s="5" t="n"/>
+      <c r="E71" s="4" t="n">
+        <v>456856.3119</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1624,6 +2082,12 @@
         <v>450737.5206</v>
       </c>
       <c r="D72" s="5" t="n"/>
+      <c r="E72" s="4" t="n">
+        <v>450737.5206</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -1640,6 +2104,12 @@
         <v>406654.2213</v>
       </c>
       <c r="D73" s="5" t="n"/>
+      <c r="E73" s="4" t="n">
+        <v>406654.2213</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1656,6 +2126,12 @@
         <v>391965.0651</v>
       </c>
       <c r="D74" s="5" t="n"/>
+      <c r="E74" s="4" t="n">
+        <v>391965.0651</v>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1672,6 +2148,12 @@
         <v>373610.2211</v>
       </c>
       <c r="D75" s="5" t="n"/>
+      <c r="E75" s="4" t="n">
+        <v>373610.2211</v>
+      </c>
+      <c r="F75" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -1688,6 +2170,12 @@
         <v>372035.7101</v>
       </c>
       <c r="D76" s="5" t="n"/>
+      <c r="E76" s="4" t="n">
+        <v>372035.7101</v>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -1704,6 +2192,12 @@
         <v>368779.171</v>
       </c>
       <c r="D77" s="5" t="n"/>
+      <c r="E77" s="4" t="n">
+        <v>368779.171</v>
+      </c>
+      <c r="F77" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -1720,6 +2214,12 @@
         <v>364313.8869</v>
       </c>
       <c r="D78" s="5" t="n"/>
+      <c r="E78" s="4" t="n">
+        <v>364313.8869</v>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -1736,6 +2236,12 @@
         <v>349130.2568</v>
       </c>
       <c r="D79" s="5" t="n"/>
+      <c r="E79" s="4" t="n">
+        <v>349130.2568</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1752,6 +2258,12 @@
         <v>317618.675</v>
       </c>
       <c r="D80" s="5" t="n"/>
+      <c r="E80" s="4" t="n">
+        <v>317618.675</v>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -1768,6 +2280,12 @@
         <v>306593.6026</v>
       </c>
       <c r="D81" s="5" t="n"/>
+      <c r="E81" s="4" t="n">
+        <v>306593.6026</v>
+      </c>
+      <c r="F81" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1784,6 +2302,12 @@
         <v>304779.1145</v>
       </c>
       <c r="D82" s="5" t="n"/>
+      <c r="E82" s="4" t="n">
+        <v>304779.1145</v>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1800,6 +2324,12 @@
         <v>279571.178</v>
       </c>
       <c r="D83" s="5" t="n"/>
+      <c r="E83" s="4" t="n">
+        <v>279571.178</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1816,6 +2346,12 @@
         <v>276846.4217</v>
       </c>
       <c r="D84" s="5" t="n"/>
+      <c r="E84" s="4" t="n">
+        <v>276846.4217</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -1832,6 +2368,12 @@
         <v>270452.3185</v>
       </c>
       <c r="D85" s="5" t="n"/>
+      <c r="E85" s="4" t="n">
+        <v>270452.3185</v>
+      </c>
+      <c r="F85" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1848,6 +2390,12 @@
         <v>265595.8775</v>
       </c>
       <c r="D86" s="5" t="n"/>
+      <c r="E86" s="4" t="n">
+        <v>265595.8775</v>
+      </c>
+      <c r="F86" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -1864,6 +2412,12 @@
         <v>262311.5799</v>
       </c>
       <c r="D87" s="5" t="n"/>
+      <c r="E87" s="4" t="n">
+        <v>262311.5799</v>
+      </c>
+      <c r="F87" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1880,6 +2434,12 @@
         <v>253086.7083</v>
       </c>
       <c r="D88" s="5" t="n"/>
+      <c r="E88" s="4" t="n">
+        <v>253086.7083</v>
+      </c>
+      <c r="F88" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -1896,6 +2456,12 @@
         <v>248683.7198</v>
       </c>
       <c r="D89" s="5" t="n"/>
+      <c r="E89" s="4" t="n">
+        <v>248683.7198</v>
+      </c>
+      <c r="F89" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1912,6 +2478,12 @@
         <v>245600</v>
       </c>
       <c r="D90" s="5" t="n"/>
+      <c r="E90" s="4" t="n">
+        <v>245600</v>
+      </c>
+      <c r="F90" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1928,6 +2500,12 @@
         <v>234392.5508</v>
       </c>
       <c r="D91" s="5" t="n"/>
+      <c r="E91" s="4" t="n">
+        <v>234392.5508</v>
+      </c>
+      <c r="F91" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1944,6 +2522,12 @@
         <v>232105.4869</v>
       </c>
       <c r="D92" s="5" t="n"/>
+      <c r="E92" s="4" t="n">
+        <v>232105.4869</v>
+      </c>
+      <c r="F92" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1960,6 +2544,12 @@
         <v>232010.2351</v>
       </c>
       <c r="D93" s="5" t="n"/>
+      <c r="E93" s="4" t="n">
+        <v>232010.2351</v>
+      </c>
+      <c r="F93" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -1976,6 +2566,12 @@
         <v>210417.5518</v>
       </c>
       <c r="D94" s="5" t="n"/>
+      <c r="E94" s="4" t="n">
+        <v>210417.5518</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -1992,6 +2588,12 @@
         <v>208196.4767</v>
       </c>
       <c r="D95" s="5" t="n"/>
+      <c r="E95" s="4" t="n">
+        <v>208196.4767</v>
+      </c>
+      <c r="F95" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2008,6 +2610,12 @@
         <v>200680.3037</v>
       </c>
       <c r="D96" s="5" t="n"/>
+      <c r="E96" s="4" t="n">
+        <v>200680.3037</v>
+      </c>
+      <c r="F96" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2024,6 +2632,12 @@
         <v>200000</v>
       </c>
       <c r="D97" s="5" t="n"/>
+      <c r="E97" s="4" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F97" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2040,6 +2654,12 @@
         <v>193698.4706</v>
       </c>
       <c r="D98" s="5" t="n"/>
+      <c r="E98" s="4" t="n">
+        <v>193698.4706</v>
+      </c>
+      <c r="F98" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2056,6 +2676,12 @@
         <v>189214.5731</v>
       </c>
       <c r="D99" s="5" t="n"/>
+      <c r="E99" s="4" t="n">
+        <v>189214.5731</v>
+      </c>
+      <c r="F99" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2072,6 +2698,12 @@
         <v>184057.6874</v>
       </c>
       <c r="D100" s="5" t="n"/>
+      <c r="E100" s="4" t="n">
+        <v>184057.6874</v>
+      </c>
+      <c r="F100" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2088,6 +2720,12 @@
         <v>179226.4255</v>
       </c>
       <c r="D101" s="5" t="n"/>
+      <c r="E101" s="4" t="n">
+        <v>179226.4255</v>
+      </c>
+      <c r="F101" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2100,13 +2738,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2130,6 +2770,16 @@
           <t>Chênh lệch</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>05/08/2026 15:59</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Chênh lệch</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2146,6 +2796,12 @@
         <v>27004519.2645</v>
       </c>
       <c r="D2" s="5" t="n"/>
+      <c r="E2" s="4" t="n">
+        <v>27004519.2645</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2162,6 +2818,12 @@
         <v>26470000</v>
       </c>
       <c r="D3" s="5" t="n"/>
+      <c r="E3" s="4" t="n">
+        <v>26470000</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2178,6 +2840,12 @@
         <v>23480366.3071</v>
       </c>
       <c r="D4" s="5" t="n"/>
+      <c r="E4" s="4" t="n">
+        <v>23480366.3071</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2194,6 +2862,12 @@
         <v>23069630.0654</v>
       </c>
       <c r="D5" s="5" t="n"/>
+      <c r="E5" s="4" t="n">
+        <v>23069630.0654</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2210,6 +2884,12 @@
         <v>21968454.2781</v>
       </c>
       <c r="D6" s="5" t="n"/>
+      <c r="E6" s="4" t="n">
+        <v>22585099.5716</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>616645.2935</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2226,6 +2906,12 @@
         <v>20000000.0069</v>
       </c>
       <c r="D7" s="5" t="n"/>
+      <c r="E7" s="4" t="n">
+        <v>20000000.0069</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2242,6 +2928,12 @@
         <v>18754869.6112</v>
       </c>
       <c r="D8" s="5" t="n"/>
+      <c r="E8" s="4" t="n">
+        <v>18754869.6112</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2258,6 +2950,12 @@
         <v>17900000</v>
       </c>
       <c r="D9" s="5" t="n"/>
+      <c r="E9" s="4" t="n">
+        <v>17900000</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2274,6 +2972,12 @@
         <v>16000000</v>
       </c>
       <c r="D10" s="5" t="n"/>
+      <c r="E10" s="4" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2290,6 +2994,12 @@
         <v>15566890.7147</v>
       </c>
       <c r="D11" s="5" t="n"/>
+      <c r="E11" s="4" t="n">
+        <v>15566890.7147</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2306,6 +3016,12 @@
         <v>15077130.0016</v>
       </c>
       <c r="D12" s="5" t="n"/>
+      <c r="E12" s="4" t="n">
+        <v>15077130.0016</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2322,6 +3038,12 @@
         <v>14000000.0458</v>
       </c>
       <c r="D13" s="5" t="n"/>
+      <c r="E13" s="4" t="n">
+        <v>14000000.0458</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2338,6 +3060,12 @@
         <v>13946038.6243</v>
       </c>
       <c r="D14" s="5" t="n"/>
+      <c r="E14" s="4" t="n">
+        <v>13946038.6243</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2354,6 +3082,12 @@
         <v>13561030.1654</v>
       </c>
       <c r="D15" s="5" t="n"/>
+      <c r="E15" s="4" t="n">
+        <v>13561030.1654</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2370,6 +3104,12 @@
         <v>13000000</v>
       </c>
       <c r="D16" s="5" t="n"/>
+      <c r="E16" s="4" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2386,6 +3126,12 @@
         <v>12877042.1771</v>
       </c>
       <c r="D17" s="5" t="n"/>
+      <c r="E17" s="4" t="n">
+        <v>12877042.1771</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2402,6 +3148,12 @@
         <v>12076398.0324</v>
       </c>
       <c r="D18" s="5" t="n"/>
+      <c r="E18" s="4" t="n">
+        <v>12076398.0324</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2418,6 +3170,12 @@
         <v>12035369.0946</v>
       </c>
       <c r="D19" s="5" t="n"/>
+      <c r="E19" s="4" t="n">
+        <v>12035369.0946</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2434,6 +3192,12 @@
         <v>11000100</v>
       </c>
       <c r="D20" s="5" t="n"/>
+      <c r="E20" s="4" t="n">
+        <v>11000100</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2450,6 +3214,12 @@
         <v>10537438.7702</v>
       </c>
       <c r="D21" s="5" t="n"/>
+      <c r="E21" s="4" t="n">
+        <v>10537438.7702</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2466,6 +3236,12 @@
         <v>10300500</v>
       </c>
       <c r="D22" s="5" t="n"/>
+      <c r="E22" s="4" t="n">
+        <v>9100000</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>-1200500</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2482,6 +3258,12 @@
         <v>10145020.9338</v>
       </c>
       <c r="D23" s="5" t="n"/>
+      <c r="E23" s="4" t="n">
+        <v>10145020.9338</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2498,6 +3280,12 @@
         <v>10064319.802</v>
       </c>
       <c r="D24" s="5" t="n"/>
+      <c r="E24" s="4" t="n">
+        <v>10064319.802</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2514,6 +3302,12 @@
         <v>10050792.1674</v>
       </c>
       <c r="D25" s="5" t="n"/>
+      <c r="E25" s="4" t="n">
+        <v>10050792.1674</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2530,6 +3324,12 @@
         <v>9974153.375</v>
       </c>
       <c r="D26" s="5" t="n"/>
+      <c r="E26" s="4" t="n">
+        <v>9974153.375</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2546,6 +3346,12 @@
         <v>9950177.2448</v>
       </c>
       <c r="D27" s="5" t="n"/>
+      <c r="E27" s="4" t="n">
+        <v>9950177.2448</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2562,6 +3368,12 @@
         <v>9450000</v>
       </c>
       <c r="D28" s="5" t="n"/>
+      <c r="E28" s="4" t="n">
+        <v>9450000</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2578,6 +3390,12 @@
         <v>8928368.352</v>
       </c>
       <c r="D29" s="5" t="n"/>
+      <c r="E29" s="4" t="n">
+        <v>8928368.352</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2594,6 +3412,12 @@
         <v>8652441.2765</v>
       </c>
       <c r="D30" s="5" t="n"/>
+      <c r="E30" s="4" t="n">
+        <v>8652441.2765</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2610,6 +3434,12 @@
         <v>8363455.9946</v>
       </c>
       <c r="D31" s="5" t="n"/>
+      <c r="E31" s="4" t="n">
+        <v>8363455.9946</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2626,6 +3456,12 @@
         <v>8023815.4821</v>
       </c>
       <c r="D32" s="5" t="n"/>
+      <c r="E32" s="4" t="n">
+        <v>8023815.4821</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2642,6 +3478,12 @@
         <v>8023361.3442</v>
       </c>
       <c r="D33" s="5" t="n"/>
+      <c r="E33" s="4" t="n">
+        <v>8023361.3442</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2658,6 +3500,12 @@
         <v>8000005.5172</v>
       </c>
       <c r="D34" s="5" t="n"/>
+      <c r="E34" s="4" t="n">
+        <v>8000005.5172</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2674,6 +3522,12 @@
         <v>7000187</v>
       </c>
       <c r="D35" s="5" t="n"/>
+      <c r="E35" s="4" t="n">
+        <v>7000187</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2690,6 +3544,12 @@
         <v>6936249.5374</v>
       </c>
       <c r="D36" s="5" t="n"/>
+      <c r="E36" s="4" t="n">
+        <v>6936249.5374</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2706,6 +3566,12 @@
         <v>6850000.7835</v>
       </c>
       <c r="D37" s="5" t="n"/>
+      <c r="E37" s="4" t="n">
+        <v>6850000.7835</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2722,6 +3588,12 @@
         <v>6500000</v>
       </c>
       <c r="D38" s="5" t="n"/>
+      <c r="E38" s="4" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2738,6 +3610,12 @@
         <v>6434508.4673</v>
       </c>
       <c r="D39" s="5" t="n"/>
+      <c r="E39" s="4" t="n">
+        <v>6434508.4673</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2754,6 +3632,12 @@
         <v>6157877.2306</v>
       </c>
       <c r="D40" s="5" t="n"/>
+      <c r="E40" s="4" t="n">
+        <v>6157877.2306</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2770,6 +3654,12 @@
         <v>5674606.3075</v>
       </c>
       <c r="D41" s="5" t="n"/>
+      <c r="E41" s="4" t="n">
+        <v>5674606.3075</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2786,6 +3676,12 @@
         <v>5565141.3215</v>
       </c>
       <c r="D42" s="5" t="n"/>
+      <c r="E42" s="4" t="n">
+        <v>5565141.3215</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2802,6 +3698,12 @@
         <v>5537959.6635</v>
       </c>
       <c r="D43" s="5" t="n"/>
+      <c r="E43" s="4" t="n">
+        <v>5537959.6635</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2818,6 +3720,12 @@
         <v>5443778.7854</v>
       </c>
       <c r="D44" s="5" t="n"/>
+      <c r="E44" s="4" t="n">
+        <v>5443778.7854</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2834,6 +3742,12 @@
         <v>5249101.3481</v>
       </c>
       <c r="D45" s="5" t="n"/>
+      <c r="E45" s="4" t="n">
+        <v>5249101.3481</v>
+      </c>
+      <c r="F45" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2850,6 +3764,12 @@
         <v>5246809.5221</v>
       </c>
       <c r="D46" s="5" t="n"/>
+      <c r="E46" s="4" t="n">
+        <v>5246809.5221</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2866,6 +3786,12 @@
         <v>5229000</v>
       </c>
       <c r="D47" s="5" t="n"/>
+      <c r="E47" s="4" t="n">
+        <v>5229000</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2882,6 +3808,12 @@
         <v>5188888.88</v>
       </c>
       <c r="D48" s="5" t="n"/>
+      <c r="E48" s="4" t="n">
+        <v>5188888.88</v>
+      </c>
+      <c r="F48" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2898,6 +3830,12 @@
         <v>5003000</v>
       </c>
       <c r="D49" s="5" t="n"/>
+      <c r="E49" s="4" t="n">
+        <v>5003000</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2914,6 +3852,12 @@
         <v>5000000.0018</v>
       </c>
       <c r="D50" s="5" t="n"/>
+      <c r="E50" s="4" t="n">
+        <v>5000000.0018</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2930,6 +3874,12 @@
         <v>4664770.6328</v>
       </c>
       <c r="D51" s="5" t="n"/>
+      <c r="E51" s="4" t="n">
+        <v>4664770.6328</v>
+      </c>
+      <c r="F51" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2946,6 +3896,12 @@
         <v>4614481.0346</v>
       </c>
       <c r="D52" s="5" t="n"/>
+      <c r="E52" s="4" t="n">
+        <v>4614481.0346</v>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2962,6 +3918,12 @@
         <v>4540406.5588</v>
       </c>
       <c r="D53" s="5" t="n"/>
+      <c r="E53" s="4" t="n">
+        <v>4540406.5588</v>
+      </c>
+      <c r="F53" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2978,6 +3940,12 @@
         <v>4537210.2091</v>
       </c>
       <c r="D54" s="5" t="n"/>
+      <c r="E54" s="4" t="n">
+        <v>4537210.2091</v>
+      </c>
+      <c r="F54" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2994,6 +3962,12 @@
         <v>4521268.8043</v>
       </c>
       <c r="D55" s="5" t="n"/>
+      <c r="E55" s="4" t="n">
+        <v>4521268.8043</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3010,6 +3984,12 @@
         <v>4519500</v>
       </c>
       <c r="D56" s="5" t="n"/>
+      <c r="E56" s="4" t="n">
+        <v>4519500</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3026,6 +4006,12 @@
         <v>4426640.2635</v>
       </c>
       <c r="D57" s="5" t="n"/>
+      <c r="E57" s="4" t="n">
+        <v>4426640.2635</v>
+      </c>
+      <c r="F57" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3042,6 +4028,12 @@
         <v>4065312.1229</v>
       </c>
       <c r="D58" s="5" t="n"/>
+      <c r="E58" s="4" t="n">
+        <v>4065312.1229</v>
+      </c>
+      <c r="F58" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3058,6 +4050,12 @@
         <v>4044917.9442</v>
       </c>
       <c r="D59" s="5" t="n"/>
+      <c r="E59" s="4" t="n">
+        <v>4044917.9442</v>
+      </c>
+      <c r="F59" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3074,6 +4072,12 @@
         <v>4000014.4373</v>
       </c>
       <c r="D60" s="5" t="n"/>
+      <c r="E60" s="4" t="n">
+        <v>4000014.4373</v>
+      </c>
+      <c r="F60" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3090,6 +4094,12 @@
         <v>3927600.0561</v>
       </c>
       <c r="D61" s="5" t="n"/>
+      <c r="E61" s="4" t="n">
+        <v>3927600.0561</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3106,6 +4116,12 @@
         <v>3891798.8644</v>
       </c>
       <c r="D62" s="5" t="n"/>
+      <c r="E62" s="4" t="n">
+        <v>3891798.8644</v>
+      </c>
+      <c r="F62" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3122,6 +4138,12 @@
         <v>3806790</v>
       </c>
       <c r="D63" s="5" t="n"/>
+      <c r="E63" s="4" t="n">
+        <v>3806790</v>
+      </c>
+      <c r="F63" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3138,6 +4160,12 @@
         <v>3777387</v>
       </c>
       <c r="D64" s="5" t="n"/>
+      <c r="E64" s="4" t="n">
+        <v>3777387</v>
+      </c>
+      <c r="F64" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3154,6 +4182,12 @@
         <v>3710432.1672</v>
       </c>
       <c r="D65" s="5" t="n"/>
+      <c r="E65" s="4" t="n">
+        <v>3710432.1672</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3170,6 +4204,12 @@
         <v>3670420</v>
       </c>
       <c r="D66" s="5" t="n"/>
+      <c r="E66" s="4" t="n">
+        <v>3670420</v>
+      </c>
+      <c r="F66" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3186,6 +4226,12 @@
         <v>3651821.6602</v>
       </c>
       <c r="D67" s="5" t="n"/>
+      <c r="E67" s="4" t="n">
+        <v>3651821.6602</v>
+      </c>
+      <c r="F67" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3202,6 +4248,12 @@
         <v>3579376.119</v>
       </c>
       <c r="D68" s="5" t="n"/>
+      <c r="E68" s="4" t="n">
+        <v>3579376.119</v>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3218,6 +4270,12 @@
         <v>3534274.8743</v>
       </c>
       <c r="D69" s="5" t="n"/>
+      <c r="E69" s="4" t="n">
+        <v>3534274.8743</v>
+      </c>
+      <c r="F69" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3234,6 +4292,12 @@
         <v>3500497.764</v>
       </c>
       <c r="D70" s="5" t="n"/>
+      <c r="E70" s="4" t="n">
+        <v>3500497.764</v>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3250,6 +4314,12 @@
         <v>3487322.2855</v>
       </c>
       <c r="D71" s="5" t="n"/>
+      <c r="E71" s="4" t="n">
+        <v>3487322.2855</v>
+      </c>
+      <c r="F71" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3266,6 +4336,12 @@
         <v>3399453.366</v>
       </c>
       <c r="D72" s="5" t="n"/>
+      <c r="E72" s="4" t="n">
+        <v>3399453.366</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3282,6 +4358,12 @@
         <v>3287999.9796</v>
       </c>
       <c r="D73" s="5" t="n"/>
+      <c r="E73" s="4" t="n">
+        <v>3287999.9796</v>
+      </c>
+      <c r="F73" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3298,6 +4380,12 @@
         <v>3277153.2544</v>
       </c>
       <c r="D74" s="5" t="n"/>
+      <c r="E74" s="4" t="n">
+        <v>3277153.2544</v>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3314,6 +4402,12 @@
         <v>3217781.3694</v>
       </c>
       <c r="D75" s="5" t="n"/>
+      <c r="E75" s="4" t="n">
+        <v>3217781.3694</v>
+      </c>
+      <c r="F75" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3330,6 +4424,12 @@
         <v>3203353.2229</v>
       </c>
       <c r="D76" s="5" t="n"/>
+      <c r="E76" s="4" t="n">
+        <v>3203353.2229</v>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3346,6 +4446,12 @@
         <v>3148181.9096</v>
       </c>
       <c r="D77" s="5" t="n"/>
+      <c r="E77" s="4" t="n">
+        <v>3148181.9096</v>
+      </c>
+      <c r="F77" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3362,6 +4468,12 @@
         <v>3130293.0222</v>
       </c>
       <c r="D78" s="5" t="n"/>
+      <c r="E78" s="4" t="n">
+        <v>3130293.0222</v>
+      </c>
+      <c r="F78" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3378,6 +4490,12 @@
         <v>3100000</v>
       </c>
       <c r="D79" s="5" t="n"/>
+      <c r="E79" s="4" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="F79" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3394,6 +4512,12 @@
         <v>3032188.4799</v>
       </c>
       <c r="D80" s="5" t="n"/>
+      <c r="E80" s="4" t="n">
+        <v>3032188.4799</v>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3410,6 +4534,12 @@
         <v>2856916.0402</v>
       </c>
       <c r="D81" s="5" t="n"/>
+      <c r="E81" s="4" t="n">
+        <v>2856916.0402</v>
+      </c>
+      <c r="F81" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3426,6 +4556,12 @@
         <v>2728360.891</v>
       </c>
       <c r="D82" s="5" t="n"/>
+      <c r="E82" s="4" t="n">
+        <v>2728360.891</v>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3442,6 +4578,12 @@
         <v>2646250.8473</v>
       </c>
       <c r="D83" s="5" t="n"/>
+      <c r="E83" s="4" t="n">
+        <v>2646250.8473</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3458,6 +4600,12 @@
         <v>2603698.568</v>
       </c>
       <c r="D84" s="5" t="n"/>
+      <c r="E84" s="4" t="n">
+        <v>2603698.568</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3474,6 +4622,12 @@
         <v>2583083.2177</v>
       </c>
       <c r="D85" s="5" t="n"/>
+      <c r="E85" s="4" t="n">
+        <v>2585748.6673</v>
+      </c>
+      <c r="F85" s="7" t="n">
+        <v>2665.4496</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3490,6 +4644,12 @@
         <v>2578757.6772</v>
       </c>
       <c r="D86" s="5" t="n"/>
+      <c r="E86" s="4" t="n">
+        <v>2578757.6772</v>
+      </c>
+      <c r="F86" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3506,6 +4666,12 @@
         <v>2566060.4818</v>
       </c>
       <c r="D87" s="5" t="n"/>
+      <c r="E87" s="4" t="n">
+        <v>2566060.4818</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3522,6 +4688,12 @@
         <v>2500000</v>
       </c>
       <c r="D88" s="5" t="n"/>
+      <c r="E88" s="4" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F88" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3538,6 +4710,12 @@
         <v>2489000.3733</v>
       </c>
       <c r="D89" s="5" t="n"/>
+      <c r="E89" s="4" t="n">
+        <v>2489000.3733</v>
+      </c>
+      <c r="F89" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3554,6 +4732,12 @@
         <v>2470041.0495</v>
       </c>
       <c r="D90" s="5" t="n"/>
+      <c r="E90" s="4" t="n">
+        <v>2470041.0495</v>
+      </c>
+      <c r="F90" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3570,6 +4754,12 @@
         <v>2411374.8288</v>
       </c>
       <c r="D91" s="5" t="n"/>
+      <c r="E91" s="4" t="n">
+        <v>2411374.8288</v>
+      </c>
+      <c r="F91" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3586,6 +4776,12 @@
         <v>2384406.6695</v>
       </c>
       <c r="D92" s="5" t="n"/>
+      <c r="E92" s="4" t="n">
+        <v>2384406.6695</v>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3602,6 +4798,12 @@
         <v>2370068.8696</v>
       </c>
       <c r="D93" s="5" t="n"/>
+      <c r="E93" s="4" t="n">
+        <v>2370068.8696</v>
+      </c>
+      <c r="F93" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3618,6 +4820,12 @@
         <v>2361819.476</v>
       </c>
       <c r="D94" s="5" t="n"/>
+      <c r="E94" s="4" t="n">
+        <v>2361819.476</v>
+      </c>
+      <c r="F94" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3634,6 +4842,12 @@
         <v>2335954.4783</v>
       </c>
       <c r="D95" s="5" t="n"/>
+      <c r="E95" s="4" t="n">
+        <v>2335954.4783</v>
+      </c>
+      <c r="F95" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3650,6 +4864,12 @@
         <v>2289568.431</v>
       </c>
       <c r="D96" s="5" t="n"/>
+      <c r="E96" s="4" t="n">
+        <v>2289568.431</v>
+      </c>
+      <c r="F96" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3666,6 +4886,12 @@
         <v>2275539.2648</v>
       </c>
       <c r="D97" s="5" t="n"/>
+      <c r="E97" s="4" t="n">
+        <v>2275539.2648</v>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3682,6 +4908,12 @@
         <v>2264858.6935</v>
       </c>
       <c r="D98" s="5" t="n"/>
+      <c r="E98" s="4" t="n">
+        <v>2264858.6935</v>
+      </c>
+      <c r="F98" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3698,6 +4930,12 @@
         <v>2263684.8207</v>
       </c>
       <c r="D99" s="5" t="n"/>
+      <c r="E99" s="4" t="n">
+        <v>2263684.8207</v>
+      </c>
+      <c r="F99" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3714,6 +4952,12 @@
         <v>2227988.9889</v>
       </c>
       <c r="D100" s="5" t="n"/>
+      <c r="E100" s="4" t="n">
+        <v>2227988.9889</v>
+      </c>
+      <c r="F100" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3730,6 +4974,12 @@
         <v>2203811.7904</v>
       </c>
       <c r="D101" s="5" t="n"/>
+      <c r="E101" s="4" t="n">
+        <v>2203811.7904</v>
+      </c>
+      <c r="F101" s="6" t="n">
+        <v>-0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>